<commit_message>
Add search validation test cases
</commit_message>
<xml_diff>
--- a/src/test/java/test-cases-scenarios/Search-test-cases.xlsx
+++ b/src/test/java/test-cases-scenarios/Search-test-cases.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18420" windowHeight="4908"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
   <si>
     <t>Test Case</t>
   </si>
@@ -157,12 +158,24 @@
   <si>
     <t xml:space="preserve">E-mail:Deneme1@gmail.com Password:Deneme search: HP LP3065 </t>
   </si>
+  <si>
+    <t>E-mail:Deneme1@gmail.com Password:Deneme1 Search: XYZ123NonExistingProduct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-mail:Deneme1@gmail.com Password:Deneme search: HP </t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-mail:Deneme1@gmail.com Password:Deneme search: Hp Lp </t>
+  </si>
+  <si>
+    <t>E-mail:Deneme1@gmail.com Password:Deneme search:HP@LP3065,HP#LP3065,HP$LP3065</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,6 +186,21 @@
     <font>
       <sz val="11"/>
       <color theme="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -201,10 +229,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -213,8 +242,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -561,6 +594,10 @@
       <c r="D3" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="E3" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="3"/>
       <c r="G3" t="s">
         <v>33</v>
       </c>
@@ -578,6 +615,10 @@
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="E4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="3"/>
       <c r="G4" t="s">
         <v>33</v>
       </c>
@@ -595,6 +636,10 @@
       <c r="D5" s="2" t="s">
         <v>26</v>
       </c>
+      <c r="E5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="3"/>
       <c r="G5" t="s">
         <v>33</v>
       </c>
@@ -612,6 +657,10 @@
       <c r="D6" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="E6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="3"/>
       <c r="G6" t="s">
         <v>33</v>
       </c>
@@ -668,7 +717,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1" display="Deneme1@gmail.com&quot;, &quot;Deneme1 Search: XYZ123NonExistingProduct"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add product detail navigation test
</commit_message>
<xml_diff>
--- a/src/test/java/test-cases-scenarios/Search-test-cases.xlsx
+++ b/src/test/java/test-cases-scenarios/Search-test-cases.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18420" windowHeight="4908"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18420" windowHeight="6720"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="41">
   <si>
     <t>Test Case</t>
   </si>
@@ -169,6 +169,12 @@
   </si>
   <si>
     <t>E-mail:Deneme1@gmail.com Password:Deneme search:HP@LP3065,HP#LP3065,HP$LP3065</t>
+  </si>
+  <si>
+    <t>E-mail:Deneme1@gmail.com Password:Deneme search:""</t>
+  </si>
+  <si>
+    <t>E-mail:Deneme1@gmail.com Password:Deneme search:Iphone</t>
   </si>
 </sst>
 </file>
@@ -678,6 +684,10 @@
       <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
+      <c r="E7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="3"/>
       <c r="G7" t="s">
         <v>33</v>
       </c>
@@ -695,6 +705,10 @@
       <c r="D8" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="E8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="3"/>
       <c r="G8" t="s">
         <v>33</v>
       </c>
@@ -712,6 +726,10 @@
       <c r="D9" s="1" t="s">
         <v>30</v>
       </c>
+      <c r="E9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="3"/>
       <c r="G9" t="s">
         <v>33</v>
       </c>

</xml_diff>